<commit_message>
Bind final v5.7.1 sensitivity reports
</commit_message>
<xml_diff>
--- a/audits/evidence/v571_rc6_candidate/report/02_quality_control/Quality_Control_Data.xlsx
+++ b/audits/evidence/v571_rc6_candidate/report/02_quality_control/Quality_Control_Data.xlsx
@@ -23,14 +23,14 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">QC_Metric_Definitions!$A$1:$D$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">README!$A$1:$B$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Source_File_Inventory!$A$1:$C$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Specimen_Technical_QC!$A$1:$BV$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Specimen_Technical_QC!$A$1:$BW$36</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="249">
   <si>
     <t>Item</t>
   </si>
@@ -68,6 +68,9 @@
     <t>group</t>
   </si>
   <si>
+    <t>group_role</t>
+  </si>
+  <si>
     <t>status</t>
   </si>
   <si>
@@ -387,6 +390,12 @@
   </si>
   <si>
     <t>w1118_sv_feb_40xx0.75-9</t>
+  </si>
+  <si>
+    <t>comparison</t>
+  </si>
+  <si>
+    <t>reference</t>
   </si>
   <si>
     <t>complete</t>
@@ -1154,79 +1163,80 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:BV36"/>
+  <dimension ref="A1:BW36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="26.7109375" customWidth="1"/>
     <col min="2" max="2" width="7.7109375" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" customWidth="1"/>
-    <col min="4" max="5" width="55.7109375" customWidth="1"/>
-    <col min="6" max="6" width="13.7109375" customWidth="1"/>
-    <col min="7" max="7" width="17.7109375" customWidth="1"/>
-    <col min="8" max="8" width="20.7109375" customWidth="1"/>
-    <col min="9" max="9" width="17.7109375" customWidth="1"/>
-    <col min="10" max="10" width="19.7109375" customWidth="1"/>
-    <col min="11" max="11" width="23.7109375" customWidth="1"/>
-    <col min="12" max="12" width="19.7109375" customWidth="1"/>
-    <col min="13" max="13" width="22.7109375" customWidth="1"/>
-    <col min="14" max="15" width="20.7109375" customWidth="1"/>
-    <col min="16" max="16" width="19.7109375" customWidth="1"/>
-    <col min="17" max="17" width="24.7109375" customWidth="1"/>
-    <col min="18" max="18" width="32.7109375" customWidth="1"/>
-    <col min="19" max="20" width="26.7109375" customWidth="1"/>
-    <col min="21" max="21" width="35.7109375" customWidth="1"/>
-    <col min="22" max="22" width="24.7109375" customWidth="1"/>
-    <col min="23" max="23" width="42.7109375" customWidth="1"/>
-    <col min="24" max="24" width="24.7109375" customWidth="1"/>
-    <col min="25" max="25" width="20.7109375" customWidth="1"/>
-    <col min="26" max="26" width="22.7109375" customWidth="1"/>
-    <col min="27" max="27" width="27.7109375" customWidth="1"/>
-    <col min="28" max="28" width="23.7109375" customWidth="1"/>
-    <col min="29" max="29" width="25.7109375" customWidth="1"/>
-    <col min="30" max="30" width="23.7109375" customWidth="1"/>
-    <col min="31" max="31" width="30.7109375" customWidth="1"/>
-    <col min="32" max="32" width="29.7109375" customWidth="1"/>
-    <col min="33" max="33" width="45.7109375" customWidth="1"/>
-    <col min="34" max="34" width="49.7109375" customWidth="1"/>
-    <col min="35" max="35" width="29.7109375" customWidth="1"/>
-    <col min="36" max="36" width="37.7109375" customWidth="1"/>
-    <col min="37" max="37" width="38.7109375" customWidth="1"/>
-    <col min="38" max="38" width="36.7109375" customWidth="1"/>
-    <col min="39" max="39" width="39.7109375" customWidth="1"/>
-    <col min="40" max="40" width="25.7109375" customWidth="1"/>
-    <col min="41" max="41" width="40.7109375" customWidth="1"/>
-    <col min="42" max="42" width="44.7109375" customWidth="1"/>
-    <col min="43" max="43" width="39.7109375" customWidth="1"/>
-    <col min="44" max="44" width="31.7109375" customWidth="1"/>
-    <col min="45" max="45" width="33.7109375" customWidth="1"/>
-    <col min="46" max="47" width="34.7109375" customWidth="1"/>
-    <col min="48" max="48" width="35.7109375" customWidth="1"/>
-    <col min="49" max="49" width="41.7109375" customWidth="1"/>
-    <col min="50" max="51" width="30.7109375" customWidth="1"/>
-    <col min="52" max="52" width="24.7109375" customWidth="1"/>
-    <col min="53" max="53" width="27.7109375" customWidth="1"/>
-    <col min="54" max="55" width="21.7109375" customWidth="1"/>
-    <col min="56" max="56" width="44.7109375" customWidth="1"/>
-    <col min="57" max="57" width="21.7109375" customWidth="1"/>
-    <col min="58" max="58" width="20.7109375" customWidth="1"/>
-    <col min="59" max="59" width="30.7109375" customWidth="1"/>
-    <col min="60" max="60" width="22.7109375" customWidth="1"/>
-    <col min="61" max="61" width="26.7109375" customWidth="1"/>
-    <col min="62" max="62" width="29.7109375" customWidth="1"/>
-    <col min="63" max="63" width="32.7109375" customWidth="1"/>
-    <col min="64" max="65" width="31.7109375" customWidth="1"/>
-    <col min="66" max="66" width="34.7109375" customWidth="1"/>
-    <col min="67" max="67" width="22.7109375" customWidth="1"/>
-    <col min="68" max="68" width="45.7109375" customWidth="1"/>
-    <col min="69" max="69" width="37.7109375" customWidth="1"/>
-    <col min="70" max="70" width="39.7109375" customWidth="1"/>
-    <col min="71" max="71" width="35.7109375" customWidth="1"/>
-    <col min="72" max="72" width="21.7109375" customWidth="1"/>
-    <col min="73" max="73" width="55.7109375" customWidth="1"/>
-    <col min="74" max="74" width="9.7109375" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" customWidth="1"/>
+    <col min="5" max="6" width="55.7109375" customWidth="1"/>
+    <col min="7" max="7" width="13.7109375" customWidth="1"/>
+    <col min="8" max="8" width="17.7109375" customWidth="1"/>
+    <col min="9" max="9" width="20.7109375" customWidth="1"/>
+    <col min="10" max="10" width="17.7109375" customWidth="1"/>
+    <col min="11" max="11" width="19.7109375" customWidth="1"/>
+    <col min="12" max="12" width="23.7109375" customWidth="1"/>
+    <col min="13" max="13" width="19.7109375" customWidth="1"/>
+    <col min="14" max="14" width="22.7109375" customWidth="1"/>
+    <col min="15" max="16" width="20.7109375" customWidth="1"/>
+    <col min="17" max="17" width="19.7109375" customWidth="1"/>
+    <col min="18" max="18" width="24.7109375" customWidth="1"/>
+    <col min="19" max="19" width="32.7109375" customWidth="1"/>
+    <col min="20" max="21" width="26.7109375" customWidth="1"/>
+    <col min="22" max="22" width="35.7109375" customWidth="1"/>
+    <col min="23" max="23" width="24.7109375" customWidth="1"/>
+    <col min="24" max="24" width="42.7109375" customWidth="1"/>
+    <col min="25" max="25" width="24.7109375" customWidth="1"/>
+    <col min="26" max="26" width="20.7109375" customWidth="1"/>
+    <col min="27" max="27" width="22.7109375" customWidth="1"/>
+    <col min="28" max="28" width="27.7109375" customWidth="1"/>
+    <col min="29" max="29" width="23.7109375" customWidth="1"/>
+    <col min="30" max="30" width="25.7109375" customWidth="1"/>
+    <col min="31" max="31" width="23.7109375" customWidth="1"/>
+    <col min="32" max="32" width="30.7109375" customWidth="1"/>
+    <col min="33" max="33" width="29.7109375" customWidth="1"/>
+    <col min="34" max="34" width="45.7109375" customWidth="1"/>
+    <col min="35" max="35" width="49.7109375" customWidth="1"/>
+    <col min="36" max="36" width="29.7109375" customWidth="1"/>
+    <col min="37" max="37" width="37.7109375" customWidth="1"/>
+    <col min="38" max="38" width="38.7109375" customWidth="1"/>
+    <col min="39" max="39" width="36.7109375" customWidth="1"/>
+    <col min="40" max="40" width="39.7109375" customWidth="1"/>
+    <col min="41" max="41" width="25.7109375" customWidth="1"/>
+    <col min="42" max="42" width="40.7109375" customWidth="1"/>
+    <col min="43" max="43" width="44.7109375" customWidth="1"/>
+    <col min="44" max="44" width="39.7109375" customWidth="1"/>
+    <col min="45" max="45" width="31.7109375" customWidth="1"/>
+    <col min="46" max="46" width="33.7109375" customWidth="1"/>
+    <col min="47" max="48" width="34.7109375" customWidth="1"/>
+    <col min="49" max="49" width="35.7109375" customWidth="1"/>
+    <col min="50" max="50" width="41.7109375" customWidth="1"/>
+    <col min="51" max="52" width="30.7109375" customWidth="1"/>
+    <col min="53" max="53" width="24.7109375" customWidth="1"/>
+    <col min="54" max="54" width="27.7109375" customWidth="1"/>
+    <col min="55" max="56" width="21.7109375" customWidth="1"/>
+    <col min="57" max="57" width="44.7109375" customWidth="1"/>
+    <col min="58" max="58" width="21.7109375" customWidth="1"/>
+    <col min="59" max="59" width="20.7109375" customWidth="1"/>
+    <col min="60" max="60" width="30.7109375" customWidth="1"/>
+    <col min="61" max="61" width="22.7109375" customWidth="1"/>
+    <col min="62" max="62" width="26.7109375" customWidth="1"/>
+    <col min="63" max="63" width="29.7109375" customWidth="1"/>
+    <col min="64" max="64" width="32.7109375" customWidth="1"/>
+    <col min="65" max="66" width="31.7109375" customWidth="1"/>
+    <col min="67" max="67" width="34.7109375" customWidth="1"/>
+    <col min="68" max="68" width="22.7109375" customWidth="1"/>
+    <col min="69" max="69" width="45.7109375" customWidth="1"/>
+    <col min="70" max="70" width="37.7109375" customWidth="1"/>
+    <col min="71" max="71" width="39.7109375" customWidth="1"/>
+    <col min="72" max="72" width="35.7109375" customWidth="1"/>
+    <col min="73" max="73" width="21.7109375" customWidth="1"/>
+    <col min="74" max="74" width="55.7109375" customWidth="1"/>
+    <col min="75" max="75" width="9.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:74">
+    <row r="1" spans="1:75">
       <c r="A1" t="s">
         <v>10</v>
       </c>
@@ -1449,79 +1459,82 @@
       <c r="BV1" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="2" spans="1:74">
+      <c r="BW1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="1:75">
       <c r="A2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B2" t="s">
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E2" t="s">
-        <v>156</v>
-      </c>
-      <c r="F2">
+        <v>124</v>
+      </c>
+      <c r="F2" t="s">
+        <v>159</v>
+      </c>
+      <c r="G2">
         <v>88</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>0.37841796875</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>0.34618410700236</v>
       </c>
-      <c r="I2">
+      <c r="J2">
         <v>318768</v>
       </c>
-      <c r="J2">
+      <c r="K2">
         <v>1048576</v>
       </c>
-      <c r="K2">
+      <c r="L2">
         <v>0.3040008544921875</v>
       </c>
-      <c r="L2">
+      <c r="M2">
         <v>45647.62830734253</v>
       </c>
-      <c r="M2">
+      <c r="N2">
         <v>88</v>
       </c>
-      <c r="N2">
+      <c r="O2">
         <v>0.34618410700236</v>
       </c>
-      <c r="O2">
+      <c r="P2">
         <v>30.46420141620768</v>
       </c>
-      <c r="P2">
+      <c r="Q2">
         <v>30.11801730920532</v>
       </c>
-      <c r="Q2">
+      <c r="R2">
         <v>1390618.542927066</v>
       </c>
-      <c r="R2">
+      <c r="S2">
         <v>88</v>
       </c>
-      <c r="S2">
+      <c r="T2">
         <v>0</v>
       </c>
-      <c r="T2">
+      <c r="U2">
         <v>87</v>
       </c>
-      <c r="U2">
+      <c r="V2">
         <v>1</v>
       </c>
-      <c r="V2">
+      <c r="W2">
         <v>26651</v>
       </c>
-      <c r="W2">
+      <c r="X2">
         <v>6.634567533020291</v>
-      </c>
-      <c r="X2">
-        <v>0</v>
       </c>
       <c r="Y2">
         <v>0</v>
@@ -1533,13 +1546,13 @@
         <v>0</v>
       </c>
       <c r="AB2">
-        <v>26651</v>
+        <v>0</v>
       </c>
       <c r="AC2">
         <v>26651</v>
       </c>
       <c r="AD2">
-        <v>0</v>
+        <v>26651</v>
       </c>
       <c r="AE2">
         <v>0</v>
@@ -1557,123 +1570,126 @@
         <v>0</v>
       </c>
       <c r="AJ2">
+        <v>0</v>
+      </c>
+      <c r="AK2">
         <v>26651</v>
-      </c>
-      <c r="AK2">
-        <v>0.9422</v>
       </c>
       <c r="AL2">
         <v>0.9422</v>
       </c>
       <c r="AM2">
+        <v>0.9422</v>
+      </c>
+      <c r="AN2">
         <v>0</v>
       </c>
-      <c r="AN2">
+      <c r="AO2">
         <v>5517</v>
       </c>
-      <c r="AO2">
+      <c r="AP2">
         <v>0</v>
       </c>
-      <c r="AP2">
+      <c r="AQ2">
         <v>5517</v>
       </c>
-      <c r="AQ2">
+      <c r="AR2">
         <v>1</v>
       </c>
-      <c r="AR2">
+      <c r="AS2">
         <v>120.8606055686923</v>
       </c>
-      <c r="AS2">
+      <c r="AT2">
         <v>396.7299320191325</v>
       </c>
-      <c r="AT2">
+      <c r="AU2">
         <v>249</v>
       </c>
-      <c r="AU2">
+      <c r="AV2">
         <v>0</v>
       </c>
-      <c r="AV2">
+      <c r="AW2">
         <v>5766</v>
       </c>
-      <c r="AW2">
+      <c r="AX2">
         <v>5517</v>
       </c>
-      <c r="AX2">
+      <c r="AY2">
         <v>53</v>
       </c>
-      <c r="AY2">
+      <c r="AZ2">
         <v>253</v>
       </c>
-      <c r="AZ2">
+      <c r="BA2">
         <v>306</v>
       </c>
-      <c r="BA2">
+      <c r="BB2">
         <v>0.0530697190426638</v>
-      </c>
-      <c r="BB2" t="b">
-        <v>1</v>
       </c>
       <c r="BC2" t="b">
         <v>1</v>
       </c>
-      <c r="BD2" t="s">
-        <v>158</v>
-      </c>
-      <c r="BE2">
+      <c r="BD2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BE2" t="s">
+        <v>161</v>
+      </c>
+      <c r="BF2">
         <v>9.92</v>
       </c>
-      <c r="BF2">
+      <c r="BG2">
         <v>1.514</v>
       </c>
-      <c r="BG2">
+      <c r="BH2">
         <v>5.322</v>
       </c>
-      <c r="BH2">
+      <c r="BI2">
         <v>1.5523</v>
       </c>
-      <c r="BI2">
+      <c r="BJ2">
         <v>1.6923</v>
       </c>
-      <c r="BJ2">
+      <c r="BK2">
         <v>1.5658</v>
       </c>
-      <c r="BK2">
+      <c r="BL2">
         <v>7.045072686098327</v>
       </c>
-      <c r="BL2">
+      <c r="BM2">
         <v>0.7806779046583288</v>
-      </c>
-      <c r="BM2">
-        <v>10.19698420605453</v>
       </c>
       <c r="BN2">
         <v>10.19698420605453</v>
       </c>
       <c r="BO2">
+        <v>10.19698420605453</v>
+      </c>
+      <c r="BP2">
         <v>1.132361996650914</v>
-      </c>
-      <c r="BP2">
-        <v>1.262565868114934</v>
       </c>
       <c r="BQ2">
         <v>1.262565868114934</v>
       </c>
       <c r="BR2">
-        <v>13.03786184729598</v>
+        <v>1.262565868114934</v>
       </c>
       <c r="BS2">
         <v>13.03786184729598</v>
       </c>
       <c r="BT2">
+        <v>13.03786184729598</v>
+      </c>
+      <c r="BU2">
         <v>0.69236821400472</v>
       </c>
-      <c r="BU2" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="3" spans="1:74">
+      <c r="BV2" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3" spans="1:75">
       <c r="A3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
@@ -1682,12 +1698,15 @@
         <v>120</v>
       </c>
       <c r="D3" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="4" spans="1:74">
+        <v>123</v>
+      </c>
+      <c r="E3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="4" spans="1:75">
       <c r="A4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B4" t="s">
         <v>7</v>
@@ -1698,10 +1717,13 @@
       <c r="D4" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="5" spans="1:74">
+      <c r="E4" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="5" spans="1:75">
       <c r="A5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B5" t="s">
         <v>7</v>
@@ -1710,12 +1732,15 @@
         <v>120</v>
       </c>
       <c r="D5" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="6" spans="1:74">
+        <v>123</v>
+      </c>
+      <c r="E5" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="6" spans="1:75">
       <c r="A6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B6" t="s">
         <v>7</v>
@@ -1724,12 +1749,15 @@
         <v>120</v>
       </c>
       <c r="D6" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="7" spans="1:74">
+        <v>123</v>
+      </c>
+      <c r="E6" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="7" spans="1:75">
       <c r="A7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B7" t="s">
         <v>7</v>
@@ -1738,12 +1766,15 @@
         <v>120</v>
       </c>
       <c r="D7" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="8" spans="1:74">
+        <v>123</v>
+      </c>
+      <c r="E7" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="8" spans="1:75">
       <c r="A8" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B8" t="s">
         <v>7</v>
@@ -1752,12 +1783,15 @@
         <v>120</v>
       </c>
       <c r="D8" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="9" spans="1:74">
+        <v>123</v>
+      </c>
+      <c r="E8" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="9" spans="1:75">
       <c r="A9" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B9" t="s">
         <v>7</v>
@@ -1766,12 +1800,15 @@
         <v>120</v>
       </c>
       <c r="D9" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="10" spans="1:74">
+        <v>123</v>
+      </c>
+      <c r="E9" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="10" spans="1:75">
       <c r="A10" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B10" t="s">
         <v>7</v>
@@ -1780,12 +1817,15 @@
         <v>120</v>
       </c>
       <c r="D10" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="11" spans="1:74">
+        <v>123</v>
+      </c>
+      <c r="E10" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="11" spans="1:75">
       <c r="A11" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B11" t="s">
         <v>7</v>
@@ -1794,12 +1834,15 @@
         <v>120</v>
       </c>
       <c r="D11" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="12" spans="1:74">
+        <v>123</v>
+      </c>
+      <c r="E11" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="12" spans="1:75">
       <c r="A12" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B12" t="s">
         <v>7</v>
@@ -1808,12 +1851,15 @@
         <v>120</v>
       </c>
       <c r="D12" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="13" spans="1:74">
+        <v>123</v>
+      </c>
+      <c r="E12" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="13" spans="1:75">
       <c r="A13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B13" t="s">
         <v>7</v>
@@ -1822,12 +1868,15 @@
         <v>120</v>
       </c>
       <c r="D13" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="14" spans="1:74">
+        <v>123</v>
+      </c>
+      <c r="E13" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="14" spans="1:75">
       <c r="A14" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B14" t="s">
         <v>7</v>
@@ -1836,12 +1885,15 @@
         <v>120</v>
       </c>
       <c r="D14" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="15" spans="1:74">
+        <v>123</v>
+      </c>
+      <c r="E14" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="15" spans="1:75">
       <c r="A15" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B15" t="s">
         <v>7</v>
@@ -1850,12 +1902,15 @@
         <v>120</v>
       </c>
       <c r="D15" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="16" spans="1:74">
+        <v>123</v>
+      </c>
+      <c r="E15" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="16" spans="1:75">
       <c r="A16" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B16" t="s">
         <v>7</v>
@@ -1864,12 +1919,15 @@
         <v>120</v>
       </c>
       <c r="D16" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="17" spans="1:73">
+        <v>123</v>
+      </c>
+      <c r="E16" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="17" spans="1:74">
       <c r="A17" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B17" t="s">
         <v>7</v>
@@ -1878,12 +1936,15 @@
         <v>120</v>
       </c>
       <c r="D17" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="18" spans="1:73">
+        <v>123</v>
+      </c>
+      <c r="E17" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="18" spans="1:74">
       <c r="A18" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B18" t="s">
         <v>7</v>
@@ -1892,12 +1953,15 @@
         <v>120</v>
       </c>
       <c r="D18" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="19" spans="1:73">
+        <v>123</v>
+      </c>
+      <c r="E18" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="19" spans="1:74">
       <c r="A19" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B19" t="s">
         <v>7</v>
@@ -1906,81 +1970,84 @@
         <v>120</v>
       </c>
       <c r="D19" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="20" spans="1:73">
+        <v>123</v>
+      </c>
+      <c r="E19" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="20" spans="1:74">
       <c r="A20" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B20" t="s">
         <v>6</v>
       </c>
       <c r="C20" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D20" t="s">
-        <v>139</v>
+        <v>122</v>
       </c>
       <c r="E20" t="s">
-        <v>157</v>
-      </c>
-      <c r="F20">
+        <v>142</v>
+      </c>
+      <c r="F20" t="s">
+        <v>160</v>
+      </c>
+      <c r="G20">
         <v>67</v>
       </c>
-      <c r="G20">
+      <c r="H20">
         <v>0.37841796875</v>
       </c>
-      <c r="H20">
+      <c r="I20">
         <v>0.3461841070023603</v>
       </c>
-      <c r="I20">
+      <c r="J20">
         <v>250920</v>
       </c>
-      <c r="J20">
+      <c r="K20">
         <v>1048576</v>
       </c>
-      <c r="K20">
+      <c r="L20">
         <v>0.2392959594726562</v>
       </c>
-      <c r="L20">
+      <c r="M20">
         <v>35931.78391456604</v>
       </c>
-      <c r="M20">
+      <c r="N20">
         <v>67</v>
       </c>
-      <c r="N20">
+      <c r="O20">
         <v>0.3461841070023603</v>
       </c>
-      <c r="O20">
+      <c r="P20">
         <v>23.19433516915814</v>
       </c>
-      <c r="P20">
+      <c r="Q20">
         <v>22.84815106215578</v>
       </c>
-      <c r="Q20">
+      <c r="R20">
         <v>833413.8393402098</v>
       </c>
-      <c r="R20">
+      <c r="S20">
         <v>67</v>
       </c>
-      <c r="S20">
+      <c r="T20">
         <v>0</v>
       </c>
-      <c r="T20">
+      <c r="U20">
         <v>66</v>
       </c>
-      <c r="U20">
+      <c r="V20">
         <v>1</v>
       </c>
-      <c r="V20">
+      <c r="W20">
         <v>16421</v>
       </c>
-      <c r="W20">
+      <c r="X20">
         <v>6.820968110616169</v>
-      </c>
-      <c r="X20">
-        <v>0</v>
       </c>
       <c r="Y20">
         <v>0</v>
@@ -1992,13 +2059,13 @@
         <v>0</v>
       </c>
       <c r="AB20">
-        <v>16421</v>
+        <v>0</v>
       </c>
       <c r="AC20">
         <v>16421</v>
       </c>
       <c r="AD20">
-        <v>0</v>
+        <v>16421</v>
       </c>
       <c r="AE20">
         <v>0</v>
@@ -2016,346 +2083,397 @@
         <v>0</v>
       </c>
       <c r="AJ20">
+        <v>0</v>
+      </c>
+      <c r="AK20">
         <v>16421</v>
-      </c>
-      <c r="AK20">
-        <v>0.9424</v>
       </c>
       <c r="AL20">
         <v>0.9424</v>
       </c>
       <c r="AM20">
+        <v>0.9424</v>
+      </c>
+      <c r="AN20">
         <v>0</v>
       </c>
-      <c r="AN20">
+      <c r="AO20">
         <v>3423</v>
       </c>
-      <c r="AO20">
+      <c r="AP20">
         <v>0</v>
       </c>
-      <c r="AP20">
+      <c r="AQ20">
         <v>3423</v>
       </c>
-      <c r="AQ20">
+      <c r="AR20">
         <v>1</v>
       </c>
-      <c r="AR20">
+      <c r="AS20">
         <v>95.2638479664346</v>
       </c>
-      <c r="AS20">
+      <c r="AT20">
         <v>410.7203214563718</v>
       </c>
-      <c r="AT20">
+      <c r="AU20">
         <v>118</v>
       </c>
-      <c r="AU20">
+      <c r="AV20">
         <v>0</v>
       </c>
-      <c r="AV20">
+      <c r="AW20">
         <v>3541</v>
       </c>
-      <c r="AW20">
+      <c r="AX20">
         <v>3423</v>
       </c>
-      <c r="AX20">
+      <c r="AY20">
         <v>213</v>
       </c>
-      <c r="AY20">
+      <c r="AZ20">
         <v>216</v>
       </c>
-      <c r="AZ20">
+      <c r="BA20">
         <v>429</v>
       </c>
-      <c r="BA20">
+      <c r="BB20">
         <v>0.1211522168878847</v>
-      </c>
-      <c r="BB20" t="b">
-        <v>1</v>
       </c>
       <c r="BC20" t="b">
         <v>1</v>
       </c>
-      <c r="BD20" t="s">
-        <v>158</v>
-      </c>
-      <c r="BE20">
+      <c r="BD20" t="b">
+        <v>1</v>
+      </c>
+      <c r="BE20" t="s">
+        <v>161</v>
+      </c>
+      <c r="BF20">
         <v>8.536</v>
       </c>
-      <c r="BF20">
+      <c r="BG20">
         <v>1.514</v>
       </c>
-      <c r="BG20">
+      <c r="BH20">
         <v>4.1685</v>
       </c>
-      <c r="BH20">
+      <c r="BI20">
         <v>1.6921</v>
       </c>
-      <c r="BI20">
+      <c r="BJ20">
         <v>1.9247</v>
       </c>
-      <c r="BJ20">
+      <c r="BK20">
         <v>1.7534</v>
       </c>
-      <c r="BK20">
+      <c r="BL20">
         <v>5.716582874626884</v>
       </c>
-      <c r="BL20">
+      <c r="BM20">
         <v>0.7724218521764534</v>
-      </c>
-      <c r="BM20">
-        <v>8.912929321313497</v>
       </c>
       <c r="BN20">
         <v>8.912929321313497</v>
       </c>
       <c r="BO20">
+        <v>8.912929321313497</v>
+      </c>
+      <c r="BP20">
         <v>1.123739361502195</v>
-      </c>
-      <c r="BP20">
-        <v>1.281608194462744</v>
       </c>
       <c r="BQ20">
         <v>1.281608194462744</v>
       </c>
       <c r="BR20">
-        <v>11.74894774832377</v>
+        <v>1.281608194462744</v>
       </c>
       <c r="BS20">
         <v>11.74894774832377</v>
       </c>
       <c r="BT20">
+        <v>11.74894774832377</v>
+      </c>
+      <c r="BU20">
         <v>0.6923682140047207</v>
       </c>
-      <c r="BU20" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="21" spans="1:73">
+      <c r="BV20" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="21" spans="1:74">
       <c r="A21" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B21" t="s">
         <v>6</v>
       </c>
       <c r="C21" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D21" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="22" spans="1:73">
+        <v>123</v>
+      </c>
+      <c r="E21" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="22" spans="1:74">
       <c r="A22" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B22" t="s">
         <v>6</v>
       </c>
       <c r="C22" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D22" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="23" spans="1:73">
+        <v>123</v>
+      </c>
+      <c r="E22" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="23" spans="1:74">
       <c r="A23" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B23" t="s">
         <v>6</v>
       </c>
       <c r="C23" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D23" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="24" spans="1:73">
+        <v>123</v>
+      </c>
+      <c r="E23" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="24" spans="1:74">
       <c r="A24" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B24" t="s">
         <v>6</v>
       </c>
       <c r="C24" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D24" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="25" spans="1:73">
+        <v>123</v>
+      </c>
+      <c r="E24" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="25" spans="1:74">
       <c r="A25" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B25" t="s">
         <v>6</v>
       </c>
       <c r="C25" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D25" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="26" spans="1:73">
+        <v>123</v>
+      </c>
+      <c r="E25" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="26" spans="1:74">
       <c r="A26" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B26" t="s">
         <v>6</v>
       </c>
       <c r="C26" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D26" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="27" spans="1:73">
+        <v>123</v>
+      </c>
+      <c r="E26" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="27" spans="1:74">
       <c r="A27" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B27" t="s">
         <v>6</v>
       </c>
       <c r="C27" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D27" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="28" spans="1:73">
+        <v>123</v>
+      </c>
+      <c r="E27" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="28" spans="1:74">
       <c r="A28" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B28" t="s">
         <v>6</v>
       </c>
       <c r="C28" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D28" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="29" spans="1:73">
+        <v>123</v>
+      </c>
+      <c r="E28" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="29" spans="1:74">
       <c r="A29" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B29" t="s">
         <v>6</v>
       </c>
       <c r="C29" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D29" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="30" spans="1:73">
+        <v>123</v>
+      </c>
+      <c r="E29" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="30" spans="1:74">
       <c r="A30" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B30" t="s">
         <v>6</v>
       </c>
       <c r="C30" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D30" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="31" spans="1:73">
+        <v>123</v>
+      </c>
+      <c r="E30" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="31" spans="1:74">
       <c r="A31" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B31" t="s">
         <v>6</v>
       </c>
       <c r="C31" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D31" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="32" spans="1:73">
+        <v>123</v>
+      </c>
+      <c r="E31" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="32" spans="1:74">
       <c r="A32" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B32" t="s">
         <v>6</v>
       </c>
       <c r="C32" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D32" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4">
+        <v>123</v>
+      </c>
+      <c r="E32" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B33" t="s">
         <v>6</v>
       </c>
       <c r="C33" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D33" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4">
+        <v>123</v>
+      </c>
+      <c r="E33" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B34" t="s">
         <v>6</v>
       </c>
       <c r="C34" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D34" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4">
+        <v>123</v>
+      </c>
+      <c r="E34" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B35" t="s">
         <v>6</v>
       </c>
       <c r="C35" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D35" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4">
+        <v>123</v>
+      </c>
+      <c r="E35" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B36" t="s">
         <v>6</v>
       </c>
       <c r="C36" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D36" t="s">
-        <v>155</v>
+        <v>123</v>
+      </c>
+      <c r="E36" t="s">
+        <v>158</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BV36"/>
+  <autoFilter ref="A1:BW36"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2396,123 +2514,123 @@
   <sheetData>
     <row r="1" spans="1:34">
       <c r="A1" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B1" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="C1" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="D1" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="E1" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="F1" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="G1" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="H1" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="I1" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="J1" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="K1" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="L1" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="M1" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="N1" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="O1" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="P1" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="Q1" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="R1" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="S1" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="T1" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="U1" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="V1" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="W1" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="X1" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="Y1" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="Z1" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="AA1" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="AB1" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="AC1" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="AD1" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="AE1" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="AF1" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="AG1" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="AH1" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
     </row>
     <row r="2" spans="1:34">
       <c r="A2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="D2" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="E2" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="F2">
         <v>3</v>
@@ -2562,19 +2680,19 @@
     </row>
     <row r="3" spans="1:34">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B3" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="C3" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="D3" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="E3" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="F3">
         <v>3</v>
@@ -2624,19 +2742,19 @@
     </row>
     <row r="4" spans="1:34">
       <c r="A4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B4" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="C4" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="D4" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="E4" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="F4">
         <v>3</v>
@@ -2715,39 +2833,39 @@
         <v>11</v>
       </c>
       <c r="C1" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="D1" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="E1" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="F1" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="G1" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="H1" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="I1" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="J1" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="K1" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="L1" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B2" t="s">
         <v>7</v>
@@ -2785,7 +2903,7 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B3" t="s">
         <v>6</v>
@@ -2842,106 +2960,106 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="B1" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="C1" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="D1" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="E1" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F1" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C2">
         <v>0.9999999999999999</v>
       </c>
       <c r="E2" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C3">
         <v>0.9999999999999999</v>
       </c>
       <c r="E3" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C4">
         <v>0.9999999999999999</v>
       </c>
       <c r="E4" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C5">
         <v>-0.9999999999999999</v>
       </c>
       <c r="E5" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C6">
         <v>-0.9999999999999999</v>
       </c>
       <c r="E6" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C7">
         <v>-0.9999999999999999</v>
       </c>
       <c r="E7" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
   </sheetData>
@@ -2972,58 +3090,58 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B1" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="C1" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="D1" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="D2" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B3" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="C3" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="D3" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B4" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="C4" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="D4" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
     </row>
   </sheetData>
@@ -3043,109 +3161,109 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B1" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="C1" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B2" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="C2" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="B3" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="C3" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B4" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C4" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="B5" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="C5" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B6" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="C6" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="B7" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="C7" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="B8" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="C8" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="B9" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="C9" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="C10" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
   </sheetData>

</xml_diff>